<commit_message>
bloque de visualizacion y modificaciones
</commit_message>
<xml_diff>
--- a/Jupyter/Dataset.xlsx
+++ b/Jupyter/Dataset.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://estudianteccr-my.sharepoint.com/personal/scruz100_estudiantec_cr/Documents/TEC/Semestre 12 2025/Taller de comunicaciones electricas/Proyecto/Proyecto-Taller_Comunicaciones/Jupyter/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FBD1A6F2-7AED-46AD-8711-69D9212CE13F}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="8_{FBD1A6F2-7AED-46AD-8711-69D9212CE13F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{37EC9249-DD3A-4467-8590-B8B1F56A9F60}"/>
   <bookViews>
-    <workbookView xWindow="19470" yWindow="1710" windowWidth="19065" windowHeight="11715" xr2:uid="{ACC2B1C0-D2A8-4737-9219-E75674099BFA}"/>
+    <workbookView xWindow="5070" yWindow="0" windowWidth="21600" windowHeight="11235" xr2:uid="{ACC2B1C0-D2A8-4737-9219-E75674099BFA}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -91,10 +91,10 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -115,9 +115,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -155,7 +155,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -261,7 +261,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -403,7 +403,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>

</xml_diff>